<commit_message>
feat(inspection): real-time reinspection banner sync, DID validation, and lot substitution mapping
</commit_message>
<xml_diff>
--- a/standart aql.xlsx
+++ b/standart aql.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\oqc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{430CDA6E-5468-4B20-8DC6-940B1E98B050}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C50EAD-7502-4D7A-869C-20AC3C377C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{E4CEBA0D-9285-4684-A01A-1413417B3737}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="48">
   <si>
     <t>Ukuran Lot</t>
   </si>
@@ -160,6 +160,15 @@
   </si>
   <si>
     <t>Untuk pengukuran standar inspeksi ( dimensi, fungsional, dan test ) dengan syarat Lot C = 0</t>
+  </si>
+  <si>
+    <t>G-I</t>
+  </si>
+  <si>
+    <t>G-II</t>
+  </si>
+  <si>
+    <t>G-III</t>
   </si>
 </sst>
 </file>
@@ -169,7 +178,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm&quot;월&quot;\ dd&quot;일&quot;"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -239,6 +248,13 @@
       <name val="Century Gothic"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="9"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -284,7 +300,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="35">
+  <borders count="39">
     <border>
       <left/>
       <right/>
@@ -688,12 +704,203 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="double">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="hair">
+        <color indexed="64"/>
+      </top>
+      <bottom style="hair">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -721,140 +928,41 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -903,8 +1011,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr bwMode="auto">
         <a:xfrm>
-          <a:off x="1752600" y="5638800"/>
-          <a:ext cx="488950" cy="361950"/>
+          <a:off x="1754827" y="5328805"/>
+          <a:ext cx="489609" cy="356507"/>
           <a:chOff x="283" y="614"/>
           <a:chExt cx="9" cy="33"/>
         </a:xfrm>
@@ -1524,648 +1632,845 @@
     <col min="2" max="2" width="13.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3"/>
-    </row>
-    <row r="3" spans="1:5" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="4" t="s">
+      <c r="B1" s="46"/>
+    </row>
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="55" t="s">
+        <v>45</v>
+      </c>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="56" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="55" t="s">
+        <v>47</v>
+      </c>
+      <c r="J2" s="55"/>
+      <c r="K2" s="57"/>
+    </row>
+    <row r="3" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="15" t="s">
+      <c r="B3" s="50"/>
+      <c r="C3" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+      <c r="F3" s="40" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="40"/>
+      <c r="H3" s="40"/>
+      <c r="I3" s="59" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" s="59"/>
+      <c r="K3" s="60"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="16" t="s">
+      <c r="B4" s="52"/>
+      <c r="C4" s="61" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="G4" s="34"/>
+      <c r="H4" s="34"/>
+      <c r="I4" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="J4" s="62"/>
+      <c r="K4" s="63"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="16" t="s">
+      <c r="B5" s="54"/>
+      <c r="C5" s="61" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="61"/>
+      <c r="E5" s="61"/>
+      <c r="F5" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="8" t="s">
+      <c r="G5" s="34"/>
+      <c r="H5" s="34"/>
+      <c r="I5" s="62" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" s="62"/>
+      <c r="K5" s="63"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A6" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="9"/>
-      <c r="C6" s="16" t="s">
+      <c r="B6" s="54"/>
+      <c r="C6" s="61" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="61"/>
+      <c r="E6" s="61"/>
+      <c r="F6" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="16"/>
-      <c r="E6" s="16"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+      <c r="G6" s="34"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="62" t="s">
+        <v>20</v>
+      </c>
+      <c r="J6" s="62"/>
+      <c r="K6" s="63"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A7" s="41" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="11"/>
-      <c r="C7" s="16" t="s">
+      <c r="B7" s="42"/>
+      <c r="C7" s="61" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="61"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+      <c r="G7" s="34"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="62" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="62"/>
+      <c r="K7" s="63"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A8" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="11"/>
-      <c r="C8" s="16" t="s">
+      <c r="B8" s="42"/>
+      <c r="C8" s="61" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="61"/>
+      <c r="E8" s="61"/>
+      <c r="F8" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
+      <c r="I8" s="62" t="s">
+        <v>22</v>
+      </c>
+      <c r="J8" s="62"/>
+      <c r="K8" s="63"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A9" s="41" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="16" t="s">
+      <c r="B9" s="42"/>
+      <c r="C9" s="61" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="61"/>
+      <c r="E9" s="61"/>
+      <c r="F9" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="16"/>
-      <c r="E9" s="16"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+      <c r="G9" s="34"/>
+      <c r="H9" s="34"/>
+      <c r="I9" s="62" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="62"/>
+      <c r="K9" s="63"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A10" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="16" t="s">
+      <c r="B10" s="42"/>
+      <c r="C10" s="61" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="61"/>
+      <c r="E10" s="61"/>
+      <c r="F10" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="62" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="62"/>
+      <c r="K10" s="63"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A11" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="11"/>
-      <c r="C11" s="16" t="s">
+      <c r="B11" s="42"/>
+      <c r="C11" s="61" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="61"/>
+      <c r="E11" s="61"/>
+      <c r="F11" s="34" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="16"/>
-      <c r="E11" s="16"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" s="10" t="s">
+      <c r="G11" s="34"/>
+      <c r="H11" s="34"/>
+      <c r="I11" s="62" t="s">
+        <v>25</v>
+      </c>
+      <c r="J11" s="62"/>
+      <c r="K11" s="63"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A12" s="41" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="11"/>
-      <c r="C12" s="16" t="s">
+      <c r="B12" s="42"/>
+      <c r="C12" s="61" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="61"/>
+      <c r="E12" s="61"/>
+      <c r="F12" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="16"/>
-      <c r="E12" s="16"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="s">
+      <c r="G12" s="34"/>
+      <c r="H12" s="34"/>
+      <c r="I12" s="62" t="s">
+        <v>26</v>
+      </c>
+      <c r="J12" s="62"/>
+      <c r="K12" s="63"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" s="41" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="11"/>
-      <c r="C13" s="16" t="s">
+      <c r="B13" s="42"/>
+      <c r="C13" s="61" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="61"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A14" s="10" t="s">
+      <c r="G13" s="34"/>
+      <c r="H13" s="34"/>
+      <c r="I13" s="62" t="s">
+        <v>27</v>
+      </c>
+      <c r="J13" s="62"/>
+      <c r="K13" s="63"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A14" s="41" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="11"/>
-      <c r="C14" s="16" t="s">
+      <c r="B14" s="42"/>
+      <c r="C14" s="61" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="61"/>
+      <c r="E14" s="61"/>
+      <c r="F14" s="34" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="62" t="s">
+        <v>28</v>
+      </c>
+      <c r="J14" s="62"/>
+      <c r="K14" s="63"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A15" s="41" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="11"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="42"/>
+      <c r="C15" s="61" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="61"/>
+      <c r="E15" s="61"/>
+      <c r="F15" s="34" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="s">
+      <c r="G15" s="34"/>
+      <c r="H15" s="34"/>
+      <c r="I15" s="62" t="s">
+        <v>29</v>
+      </c>
+      <c r="J15" s="62"/>
+      <c r="K15" s="63"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A16" s="41" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="16" t="s">
+      <c r="B16" s="42"/>
+      <c r="C16" s="61" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="61"/>
+      <c r="E16" s="61"/>
+      <c r="F16" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-    </row>
-    <row r="17" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="12" t="s">
+      <c r="G16" s="34"/>
+      <c r="H16" s="34"/>
+      <c r="I16" s="62" t="s">
+        <v>30</v>
+      </c>
+      <c r="J16" s="62"/>
+      <c r="K16" s="63"/>
+    </row>
+    <row r="17" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A17" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="13"/>
-      <c r="C17" s="17" t="s">
+      <c r="B17" s="44"/>
+      <c r="C17" s="64" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="64"/>
+      <c r="E17" s="64"/>
+      <c r="F17" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="17"/>
-      <c r="E17" s="17"/>
-    </row>
-    <row r="19" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="20" spans="1:5" ht="39" x14ac:dyDescent="0.35">
-      <c r="A20" s="18" t="s">
+      <c r="G17" s="35"/>
+      <c r="H17" s="35"/>
+      <c r="I17" s="65" t="s">
+        <v>35</v>
+      </c>
+      <c r="J17" s="65"/>
+      <c r="K17" s="66"/>
+    </row>
+    <row r="19" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="20" spans="1:11" ht="19.5" x14ac:dyDescent="0.35">
+      <c r="A20" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="19" t="s">
+      <c r="B20" s="2" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A21" s="20" t="s">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A21" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="21" t="s">
+      <c r="B21" s="38" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A22" s="22"/>
-      <c r="B22" s="23"/>
-      <c r="C22" s="32" t="s">
+    <row r="22" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A22" s="37"/>
+      <c r="B22" s="39"/>
+      <c r="C22" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="33" t="s">
+      <c r="D22" s="12" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="15" thickTop="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="24" t="s">
+    <row r="23" spans="1:11" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="25">
+      <c r="B23" s="4">
         <v>2</v>
       </c>
-      <c r="C23" s="34"/>
-      <c r="D23" s="35"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A24" s="24" t="s">
+      <c r="C23" s="13"/>
+      <c r="D23" s="14"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B24" s="25">
+      <c r="B24" s="4">
         <v>3</v>
       </c>
-      <c r="C24" s="34"/>
-      <c r="D24" s="35"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A25" s="26" t="s">
+      <c r="C24" s="13"/>
+      <c r="D24" s="14"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B25" s="27">
+      <c r="B25" s="6">
         <v>5</v>
       </c>
-      <c r="C25" s="36"/>
-      <c r="D25" s="37"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A26" s="28" t="s">
+      <c r="C25" s="15"/>
+      <c r="D25" s="16"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B26" s="29">
+      <c r="B26" s="8">
         <v>8</v>
       </c>
-      <c r="C26" s="38"/>
-      <c r="D26" s="39"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A27" s="24" t="s">
+      <c r="C26" s="17"/>
+      <c r="D26" s="18"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A27" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="25">
+      <c r="B27" s="4">
         <v>13</v>
       </c>
-      <c r="C27" s="34"/>
-      <c r="D27" s="35"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A28" s="26" t="s">
+      <c r="C27" s="13"/>
+      <c r="D27" s="14"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B28" s="27">
+      <c r="B28" s="6">
         <v>20</v>
       </c>
-      <c r="C28" s="40"/>
-      <c r="D28" s="37"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A29" s="28" t="s">
+      <c r="C28" s="19"/>
+      <c r="D28" s="16"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A29" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="29">
+      <c r="B29" s="8">
         <v>32</v>
       </c>
-      <c r="C29" s="38">
+      <c r="C29" s="17">
         <v>0</v>
       </c>
-      <c r="D29" s="41">
+      <c r="D29" s="20">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" s="24" t="s">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A30" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B30" s="25">
+      <c r="B30" s="4">
         <v>50</v>
       </c>
-      <c r="C30" s="42"/>
-      <c r="D30" s="35"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A31" s="26" t="s">
+      <c r="C30" s="21"/>
+      <c r="D30" s="14"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B31" s="27">
+      <c r="B31" s="6">
         <v>80</v>
       </c>
-      <c r="C31" s="40"/>
-      <c r="D31" s="37"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" s="28" t="s">
+      <c r="C31" s="19"/>
+      <c r="D31" s="16"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B32" s="29">
+      <c r="B32" s="8">
         <v>125</v>
       </c>
-      <c r="C32" s="41">
+      <c r="C32" s="20">
         <v>1</v>
       </c>
-      <c r="D32" s="41">
+      <c r="D32" s="20">
         <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A33" s="24" t="s">
+      <c r="A33" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B33" s="25">
+      <c r="B33" s="4">
         <v>200</v>
       </c>
-      <c r="C33" s="42">
+      <c r="C33" s="21">
         <v>2</v>
       </c>
-      <c r="D33" s="35">
+      <c r="D33" s="14">
         <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A34" s="26" t="s">
+      <c r="A34" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B34" s="27">
+      <c r="B34" s="6">
         <v>315</v>
       </c>
-      <c r="C34" s="40">
+      <c r="C34" s="19">
         <v>3</v>
       </c>
-      <c r="D34" s="40">
+      <c r="D34" s="19">
         <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A35" s="24" t="s">
+      <c r="A35" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="25">
+      <c r="B35" s="4">
         <v>500</v>
       </c>
-      <c r="C35" s="34">
+      <c r="C35" s="13">
         <v>5</v>
       </c>
-      <c r="D35" s="35">
+      <c r="D35" s="14">
         <v>6</v>
       </c>
     </row>
     <row r="36" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A36" s="24" t="s">
+      <c r="A36" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B36" s="25">
+      <c r="B36" s="4">
         <v>800</v>
       </c>
-      <c r="C36" s="34">
+      <c r="C36" s="13">
         <v>7</v>
       </c>
-      <c r="D36" s="35">
+      <c r="D36" s="14">
         <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:53" x14ac:dyDescent="0.35">
-      <c r="A37" s="24" t="s">
+      <c r="A37" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B37" s="25">
+      <c r="B37" s="4">
         <v>1250</v>
       </c>
-      <c r="C37" s="42">
+      <c r="C37" s="21">
         <v>10</v>
       </c>
-      <c r="D37" s="42">
+      <c r="D37" s="21">
         <v>11</v>
       </c>
     </row>
     <row r="38" spans="1:53" ht="18.5" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="30" t="s">
+      <c r="A38" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="31">
+      <c r="B38" s="10">
         <v>2000</v>
       </c>
-      <c r="C38" s="43">
+      <c r="C38" s="22">
         <v>14</v>
       </c>
-      <c r="D38" s="44">
+      <c r="D38" s="23">
         <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:53" ht="18" x14ac:dyDescent="0.35">
-      <c r="A39" s="45" t="s">
+      <c r="A39" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="46"/>
-      <c r="C39" s="47" t="s">
+      <c r="B39" s="25"/>
+      <c r="C39" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="D39" s="47"/>
-      <c r="E39" s="47"/>
-      <c r="F39" s="47"/>
-      <c r="G39" s="47"/>
-      <c r="H39" s="47"/>
-      <c r="I39" s="47"/>
-      <c r="J39" s="47"/>
-      <c r="K39" s="47"/>
-      <c r="L39" s="47"/>
-      <c r="M39" s="47"/>
-      <c r="N39" s="47"/>
-      <c r="O39" s="47"/>
-      <c r="P39" s="47"/>
-      <c r="Q39" s="47"/>
-      <c r="R39" s="47"/>
-      <c r="S39" s="47"/>
-      <c r="T39" s="47"/>
-      <c r="U39" s="47"/>
-      <c r="V39" s="47"/>
-      <c r="W39" s="47"/>
-      <c r="X39" s="47"/>
-      <c r="Y39" s="47"/>
-      <c r="Z39" s="47"/>
-      <c r="AA39" s="47"/>
-      <c r="AB39" s="47"/>
-      <c r="AC39" s="47"/>
-      <c r="AD39" s="47"/>
-      <c r="AE39" s="47"/>
-      <c r="AF39" s="47"/>
-      <c r="AG39" s="47"/>
-      <c r="AH39" s="47"/>
-      <c r="AI39" s="47"/>
-      <c r="AJ39" s="47"/>
-      <c r="AK39" s="47"/>
-      <c r="AL39" s="47"/>
-      <c r="AM39" s="47"/>
-      <c r="AN39" s="47"/>
-      <c r="AO39" s="47"/>
-      <c r="AP39" s="47"/>
-      <c r="AQ39" s="47"/>
-      <c r="AR39" s="48" t="s">
+      <c r="D39" s="32"/>
+      <c r="E39" s="32"/>
+      <c r="F39" s="32"/>
+      <c r="G39" s="32"/>
+      <c r="H39" s="32"/>
+      <c r="I39" s="32"/>
+      <c r="J39" s="32"/>
+      <c r="K39" s="32"/>
+      <c r="L39" s="32"/>
+      <c r="M39" s="32"/>
+      <c r="N39" s="32"/>
+      <c r="O39" s="32"/>
+      <c r="P39" s="32"/>
+      <c r="Q39" s="32"/>
+      <c r="R39" s="32"/>
+      <c r="S39" s="32"/>
+      <c r="T39" s="32"/>
+      <c r="U39" s="32"/>
+      <c r="V39" s="32"/>
+      <c r="W39" s="32"/>
+      <c r="X39" s="32"/>
+      <c r="Y39" s="32"/>
+      <c r="Z39" s="32"/>
+      <c r="AA39" s="32"/>
+      <c r="AB39" s="32"/>
+      <c r="AC39" s="32"/>
+      <c r="AD39" s="32"/>
+      <c r="AE39" s="32"/>
+      <c r="AF39" s="32"/>
+      <c r="AG39" s="32"/>
+      <c r="AH39" s="32"/>
+      <c r="AI39" s="32"/>
+      <c r="AJ39" s="32"/>
+      <c r="AK39" s="32"/>
+      <c r="AL39" s="32"/>
+      <c r="AM39" s="32"/>
+      <c r="AN39" s="32"/>
+      <c r="AO39" s="32"/>
+      <c r="AP39" s="32"/>
+      <c r="AQ39" s="32"/>
+      <c r="AR39" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="AS39" s="49"/>
-      <c r="AT39" s="49"/>
-      <c r="AU39" s="49"/>
-      <c r="AV39" s="49"/>
-      <c r="AW39" s="49"/>
-      <c r="AX39" s="49"/>
-      <c r="AY39" s="49"/>
-      <c r="AZ39" s="49"/>
-      <c r="BA39" s="49"/>
+      <c r="AS39" s="27"/>
+      <c r="AT39" s="27"/>
+      <c r="AU39" s="27"/>
+      <c r="AV39" s="27"/>
+      <c r="AW39" s="27"/>
+      <c r="AX39" s="27"/>
+      <c r="AY39" s="27"/>
+      <c r="AZ39" s="27"/>
+      <c r="BA39" s="27"/>
     </row>
     <row r="40" spans="1:53" ht="18" x14ac:dyDescent="0.35">
-      <c r="A40" s="45" t="s">
+      <c r="A40" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B40" s="46"/>
-      <c r="C40" s="50" t="s">
+      <c r="B40" s="25"/>
+      <c r="C40" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="D40" s="50"/>
-      <c r="E40" s="50"/>
-      <c r="F40" s="50"/>
-      <c r="G40" s="50"/>
-      <c r="H40" s="50"/>
-      <c r="I40" s="50"/>
-      <c r="J40" s="50"/>
-      <c r="K40" s="50"/>
-      <c r="L40" s="50"/>
-      <c r="M40" s="50"/>
-      <c r="N40" s="50"/>
-      <c r="O40" s="50"/>
-      <c r="P40" s="50"/>
-      <c r="Q40" s="50"/>
-      <c r="R40" s="50"/>
-      <c r="S40" s="50"/>
-      <c r="T40" s="50"/>
-      <c r="U40" s="50"/>
-      <c r="V40" s="50"/>
-      <c r="W40" s="50"/>
-      <c r="X40" s="50"/>
-      <c r="Y40" s="50"/>
-      <c r="Z40" s="50"/>
-      <c r="AA40" s="50"/>
-      <c r="AB40" s="50"/>
-      <c r="AC40" s="50"/>
-      <c r="AD40" s="50"/>
-      <c r="AE40" s="50"/>
-      <c r="AF40" s="50"/>
-      <c r="AG40" s="50"/>
-      <c r="AH40" s="50"/>
-      <c r="AI40" s="50"/>
-      <c r="AJ40" s="50"/>
-      <c r="AK40" s="50"/>
-      <c r="AL40" s="50"/>
-      <c r="AM40" s="50"/>
-      <c r="AN40" s="50"/>
-      <c r="AO40" s="50"/>
-      <c r="AP40" s="50"/>
-      <c r="AQ40" s="50"/>
-      <c r="AR40" s="51" t="s">
+      <c r="D40" s="33"/>
+      <c r="E40" s="33"/>
+      <c r="F40" s="33"/>
+      <c r="G40" s="33"/>
+      <c r="H40" s="33"/>
+      <c r="I40" s="33"/>
+      <c r="J40" s="33"/>
+      <c r="K40" s="33"/>
+      <c r="L40" s="33"/>
+      <c r="M40" s="33"/>
+      <c r="N40" s="33"/>
+      <c r="O40" s="33"/>
+      <c r="P40" s="33"/>
+      <c r="Q40" s="33"/>
+      <c r="R40" s="33"/>
+      <c r="S40" s="33"/>
+      <c r="T40" s="33"/>
+      <c r="U40" s="33"/>
+      <c r="V40" s="33"/>
+      <c r="W40" s="33"/>
+      <c r="X40" s="33"/>
+      <c r="Y40" s="33"/>
+      <c r="Z40" s="33"/>
+      <c r="AA40" s="33"/>
+      <c r="AB40" s="33"/>
+      <c r="AC40" s="33"/>
+      <c r="AD40" s="33"/>
+      <c r="AE40" s="33"/>
+      <c r="AF40" s="33"/>
+      <c r="AG40" s="33"/>
+      <c r="AH40" s="33"/>
+      <c r="AI40" s="33"/>
+      <c r="AJ40" s="33"/>
+      <c r="AK40" s="33"/>
+      <c r="AL40" s="33"/>
+      <c r="AM40" s="33"/>
+      <c r="AN40" s="33"/>
+      <c r="AO40" s="33"/>
+      <c r="AP40" s="33"/>
+      <c r="AQ40" s="33"/>
+      <c r="AR40" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="AS40" s="52"/>
-      <c r="AT40" s="52"/>
-      <c r="AU40" s="52"/>
-      <c r="AV40" s="52"/>
-      <c r="AW40" s="52"/>
-      <c r="AX40" s="53"/>
-      <c r="AY40" s="53"/>
-      <c r="AZ40" s="53"/>
-      <c r="BA40" s="53"/>
+      <c r="AS40" s="29"/>
+      <c r="AT40" s="29"/>
+      <c r="AU40" s="29"/>
+      <c r="AV40" s="29"/>
+      <c r="AW40" s="29"/>
+      <c r="AX40" s="30"/>
+      <c r="AY40" s="30"/>
+      <c r="AZ40" s="30"/>
+      <c r="BA40" s="30"/>
     </row>
     <row r="41" spans="1:53" ht="18" x14ac:dyDescent="0.35">
-      <c r="A41" s="45" t="s">
+      <c r="A41" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="46" t="s">
+      <c r="B41" s="25" t="s">
         <v>43</v>
       </c>
-      <c r="C41" s="46"/>
-      <c r="D41" s="46"/>
-      <c r="E41" s="46"/>
-      <c r="F41" s="46"/>
-      <c r="G41" s="46"/>
-      <c r="H41" s="46"/>
-      <c r="I41" s="46"/>
-      <c r="J41" s="46"/>
-      <c r="K41" s="46"/>
-      <c r="L41" s="46"/>
-      <c r="M41" s="46"/>
-      <c r="N41" s="46"/>
-      <c r="O41" s="46"/>
-      <c r="P41" s="46"/>
-      <c r="Q41" s="46"/>
-      <c r="R41" s="46"/>
-      <c r="S41" s="46"/>
-      <c r="T41" s="46"/>
-      <c r="U41" s="46"/>
-      <c r="V41" s="46"/>
-      <c r="W41" s="46"/>
-      <c r="X41" s="46"/>
-      <c r="Y41" s="46"/>
-      <c r="Z41" s="46"/>
-      <c r="AA41" s="54"/>
-      <c r="AB41" s="54"/>
-      <c r="AC41" s="54"/>
-      <c r="AD41" s="54"/>
-      <c r="AE41" s="54"/>
-      <c r="AF41" s="54"/>
-      <c r="AG41" s="54"/>
-      <c r="AH41" s="54"/>
-      <c r="AI41" s="54"/>
-      <c r="AJ41" s="54"/>
-      <c r="AK41" s="54"/>
-      <c r="AL41" s="54"/>
-      <c r="AM41" s="54"/>
-      <c r="AN41" s="54"/>
-      <c r="AO41" s="54"/>
-      <c r="AP41" s="54"/>
-      <c r="AQ41" s="54"/>
-      <c r="AR41" s="54"/>
-      <c r="AS41" s="54"/>
-      <c r="AT41" s="54"/>
-      <c r="AU41" s="54"/>
-      <c r="AV41" s="54"/>
-      <c r="AW41" s="54"/>
-      <c r="AX41" s="54"/>
-      <c r="AY41" s="54"/>
-      <c r="AZ41" s="54"/>
-      <c r="BA41" s="54"/>
+      <c r="C41" s="25"/>
+      <c r="D41" s="25"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="25"/>
+      <c r="G41" s="25"/>
+      <c r="H41" s="25"/>
+      <c r="I41" s="25"/>
+      <c r="J41" s="25"/>
+      <c r="K41" s="25"/>
+      <c r="L41" s="25"/>
+      <c r="M41" s="25"/>
+      <c r="N41" s="25"/>
+      <c r="O41" s="25"/>
+      <c r="P41" s="25"/>
+      <c r="Q41" s="25"/>
+      <c r="R41" s="25"/>
+      <c r="S41" s="25"/>
+      <c r="T41" s="25"/>
+      <c r="U41" s="25"/>
+      <c r="V41" s="25"/>
+      <c r="W41" s="25"/>
+      <c r="X41" s="25"/>
+      <c r="Y41" s="25"/>
+      <c r="Z41" s="25"/>
+      <c r="AA41" s="31"/>
+      <c r="AB41" s="31"/>
+      <c r="AC41" s="31"/>
+      <c r="AD41" s="31"/>
+      <c r="AE41" s="31"/>
+      <c r="AF41" s="31"/>
+      <c r="AG41" s="31"/>
+      <c r="AH41" s="31"/>
+      <c r="AI41" s="31"/>
+      <c r="AJ41" s="31"/>
+      <c r="AK41" s="31"/>
+      <c r="AL41" s="31"/>
+      <c r="AM41" s="31"/>
+      <c r="AN41" s="31"/>
+      <c r="AO41" s="31"/>
+      <c r="AP41" s="31"/>
+      <c r="AQ41" s="31"/>
+      <c r="AR41" s="31"/>
+      <c r="AS41" s="31"/>
+      <c r="AT41" s="31"/>
+      <c r="AU41" s="31"/>
+      <c r="AV41" s="31"/>
+      <c r="AW41" s="31"/>
+      <c r="AX41" s="31"/>
+      <c r="AY41" s="31"/>
+      <c r="AZ41" s="31"/>
+      <c r="BA41" s="31"/>
     </row>
     <row r="42" spans="1:53" ht="18" x14ac:dyDescent="0.35">
-      <c r="A42" s="45" t="s">
+      <c r="A42" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B42" s="46" t="s">
+      <c r="B42" s="25" t="s">
         <v>44</v>
       </c>
-      <c r="C42" s="46"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="46"/>
-      <c r="F42" s="46"/>
-      <c r="G42" s="46"/>
-      <c r="H42" s="46"/>
-      <c r="I42" s="46"/>
-      <c r="J42" s="46"/>
-      <c r="K42" s="46"/>
-      <c r="L42" s="46"/>
-      <c r="M42" s="46"/>
-      <c r="N42" s="46"/>
-      <c r="O42" s="46"/>
-      <c r="P42" s="46"/>
-      <c r="Q42" s="46"/>
-      <c r="R42" s="46"/>
-      <c r="S42" s="46"/>
-      <c r="T42" s="46"/>
-      <c r="U42" s="46"/>
-      <c r="V42" s="46"/>
-      <c r="W42" s="46"/>
-      <c r="X42" s="46"/>
-      <c r="Y42" s="46"/>
-      <c r="Z42" s="46"/>
-      <c r="AA42" s="54"/>
-      <c r="AB42" s="54"/>
-      <c r="AC42" s="54"/>
-      <c r="AD42" s="54"/>
-      <c r="AE42" s="54"/>
-      <c r="AF42" s="54"/>
-      <c r="AG42" s="54"/>
-      <c r="AH42" s="54"/>
-      <c r="AI42" s="54"/>
-      <c r="AJ42" s="54"/>
-      <c r="AK42" s="54"/>
-      <c r="AL42" s="54"/>
-      <c r="AM42" s="54"/>
-      <c r="AN42" s="54"/>
-      <c r="AO42" s="54"/>
-      <c r="AP42" s="54"/>
-      <c r="AQ42" s="54"/>
-      <c r="AR42" s="54"/>
-      <c r="AS42" s="54"/>
-      <c r="AT42" s="54"/>
-      <c r="AU42" s="54"/>
-      <c r="AV42" s="54"/>
-      <c r="AW42" s="54"/>
-      <c r="AX42" s="54"/>
-      <c r="AY42" s="54"/>
-      <c r="AZ42" s="54"/>
-      <c r="BA42" s="54"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="25"/>
+      <c r="G42" s="25"/>
+      <c r="H42" s="25"/>
+      <c r="I42" s="25"/>
+      <c r="J42" s="25"/>
+      <c r="K42" s="25"/>
+      <c r="L42" s="25"/>
+      <c r="M42" s="25"/>
+      <c r="N42" s="25"/>
+      <c r="O42" s="25"/>
+      <c r="P42" s="25"/>
+      <c r="Q42" s="25"/>
+      <c r="R42" s="25"/>
+      <c r="S42" s="25"/>
+      <c r="T42" s="25"/>
+      <c r="U42" s="25"/>
+      <c r="V42" s="25"/>
+      <c r="W42" s="25"/>
+      <c r="X42" s="25"/>
+      <c r="Y42" s="25"/>
+      <c r="Z42" s="25"/>
+      <c r="AA42" s="31"/>
+      <c r="AB42" s="31"/>
+      <c r="AC42" s="31"/>
+      <c r="AD42" s="31"/>
+      <c r="AE42" s="31"/>
+      <c r="AF42" s="31"/>
+      <c r="AG42" s="31"/>
+      <c r="AH42" s="31"/>
+      <c r="AI42" s="31"/>
+      <c r="AJ42" s="31"/>
+      <c r="AK42" s="31"/>
+      <c r="AL42" s="31"/>
+      <c r="AM42" s="31"/>
+      <c r="AN42" s="31"/>
+      <c r="AO42" s="31"/>
+      <c r="AP42" s="31"/>
+      <c r="AQ42" s="31"/>
+      <c r="AR42" s="31"/>
+      <c r="AS42" s="31"/>
+      <c r="AT42" s="31"/>
+      <c r="AU42" s="31"/>
+      <c r="AV42" s="31"/>
+      <c r="AW42" s="31"/>
+      <c r="AX42" s="31"/>
+      <c r="AY42" s="31"/>
+      <c r="AZ42" s="31"/>
+      <c r="BA42" s="31"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="C39:AQ39"/>
-    <mergeCell ref="C40:AQ40"/>
-    <mergeCell ref="C14:E14"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="C17:E17"/>
+  <mergeCells count="68">
+    <mergeCell ref="F11:H11"/>
+    <mergeCell ref="I11:K11"/>
+    <mergeCell ref="F12:H12"/>
+    <mergeCell ref="I12:K12"/>
+    <mergeCell ref="F13:H13"/>
+    <mergeCell ref="I13:K13"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="F9:H9"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="F10:H10"/>
+    <mergeCell ref="I10:K10"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C2:E2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="I2:K2"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="F6:H6"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A21:A22"/>
     <mergeCell ref="B21:B22"/>
     <mergeCell ref="C3:E3"/>
@@ -2182,19 +2487,20 @@
     <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C39:AQ39"/>
+    <mergeCell ref="C40:AQ40"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F14:H14"/>
+    <mergeCell ref="I14:K14"/>
+    <mergeCell ref="F15:H15"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="I16:K16"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="I17:K17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>